<commit_message>
Naprawa: dopisane produkty (323-333) wpisane w istniejace wiersze
Wczesniej nowe wiersze byly dodawane po istniejacych pustych wierszach
323-422, co tworzylo zduplikowane numery wierszy - Excel ignorowal
dopisane dane i plik konczyl sie na 322. Teraz dane wpisywane sa w
istniejace wiersze, bez duplikatow.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ebyH8W53QuuGWDHJXrtLV
</commit_message>
<xml_diff>
--- a/PRACTIC_PRODUCT_OFFER_2026_MERGED.xlsx
+++ b/PRACTIC_PRODUCT_OFFER_2026_MERGED.xlsx
@@ -47092,577 +47092,428 @@
       <c r="AW322" s="90"/>
       <c r="AX322" s="90"/>
     </row>
-    <row r="323" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A323" s="12"/>
-      <c r="B323" s="65"/>
-      <c r="C323" s="15"/>
-      <c r="D323" s="14"/>
-      <c r="E323" s="14"/>
-      <c r="F323" s="31"/>
-      <c r="G323" s="151"/>
-      <c r="H323" s="155"/>
-      <c r="I323" s="15"/>
-      <c r="J323" s="15"/>
-      <c r="K323" s="15"/>
-      <c r="L323" s="11"/>
-      <c r="M323" s="11"/>
-      <c r="N323" s="32"/>
-      <c r="O323" s="32"/>
-      <c r="P323" s="32"/>
-      <c r="Q323" s="90"/>
-      <c r="R323" s="90"/>
-      <c r="S323" s="90"/>
-      <c r="T323" s="90"/>
-      <c r="U323" s="90"/>
-      <c r="V323" s="90"/>
-      <c r="W323" s="90"/>
-      <c r="X323" s="90"/>
-      <c r="Y323" s="90"/>
-      <c r="Z323" s="90"/>
-      <c r="AA323" s="90"/>
-      <c r="AB323" s="90"/>
-      <c r="AC323" s="90"/>
-      <c r="AD323" s="90"/>
-      <c r="AE323" s="90"/>
-      <c r="AF323" s="90"/>
-      <c r="AG323" s="90"/>
-      <c r="AH323" s="90"/>
-      <c r="AI323" s="90"/>
-      <c r="AJ323" s="90"/>
-      <c r="AK323" s="90"/>
-      <c r="AL323" s="90"/>
-      <c r="AM323" s="90"/>
-      <c r="AN323" s="90"/>
-      <c r="AO323" s="90"/>
-      <c r="AP323" s="90"/>
-      <c r="AQ323" s="90"/>
-      <c r="AR323" s="90"/>
-      <c r="AS323" s="90"/>
-      <c r="AT323" s="90"/>
-      <c r="AU323" s="90"/>
-      <c r="AV323" s="90"/>
-      <c r="AW323" s="90"/>
-      <c r="AX323" s="90"/>
+    <row r="323" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
+      <c r="A323" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">471.</t>
+        </is>
+      </c>
+      <c r="E323" s="20">
+        <v>5903456123697.0</v>
+      </c>
+      <c r="G323" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Folding table for bed - cappuccino</t>
+        </is>
+      </c>
+      <c r="H323" s="154">
+        <v>4.2526942711287585</v>
+      </c>
+      <c r="I323" s="18">
+        <v>6.0</v>
+      </c>
+      <c r="J323" s="18">
+        <v>108.0</v>
+      </c>
+      <c r="K323" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">54x35.5x26 cm</t>
+        </is>
+      </c>
+      <c r="L323" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">970</t>
+        </is>
+      </c>
+      <c r="M323" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">polipropylen</t>
+        </is>
+      </c>
     </row>
-    <row r="324" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A324" s="12"/>
-      <c r="B324" s="65"/>
-      <c r="C324" s="15"/>
-      <c r="D324" s="14"/>
-      <c r="E324" s="14"/>
-      <c r="F324" s="31"/>
-      <c r="G324" s="151"/>
-      <c r="H324" s="155"/>
-      <c r="I324" s="15"/>
-      <c r="J324" s="15"/>
-      <c r="K324" s="15"/>
-      <c r="L324" s="11"/>
-      <c r="M324" s="11"/>
-      <c r="N324" s="32"/>
-      <c r="O324" s="32"/>
-      <c r="P324" s="32"/>
-      <c r="Q324" s="90"/>
-      <c r="R324" s="90"/>
-      <c r="S324" s="90"/>
-      <c r="T324" s="90"/>
-      <c r="U324" s="90"/>
-      <c r="V324" s="90"/>
-      <c r="W324" s="90"/>
-      <c r="X324" s="90"/>
-      <c r="Y324" s="90"/>
-      <c r="Z324" s="90"/>
-      <c r="AA324" s="90"/>
-      <c r="AB324" s="90"/>
-      <c r="AC324" s="90"/>
-      <c r="AD324" s="90"/>
-      <c r="AE324" s="90"/>
-      <c r="AF324" s="90"/>
-      <c r="AG324" s="90"/>
-      <c r="AH324" s="90"/>
-      <c r="AI324" s="90"/>
-      <c r="AJ324" s="90"/>
-      <c r="AK324" s="90"/>
-      <c r="AL324" s="90"/>
-      <c r="AM324" s="90"/>
-      <c r="AN324" s="90"/>
-      <c r="AO324" s="90"/>
-      <c r="AP324" s="90"/>
-      <c r="AQ324" s="90"/>
-      <c r="AR324" s="90"/>
-      <c r="AS324" s="90"/>
-      <c r="AT324" s="90"/>
-      <c r="AU324" s="90"/>
-      <c r="AV324" s="90"/>
-      <c r="AW324" s="90"/>
-      <c r="AX324" s="90"/>
+    <row r="324" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
+      <c r="A324" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">472.</t>
+        </is>
+      </c>
+      <c r="E324" s="20">
+        <v>5903456119478.0</v>
+      </c>
+      <c r="G324" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MINI BINI - handy container for bio waste - green color container gray cover 35% bio - 4.5L</t>
+        </is>
+      </c>
+      <c r="H324" s="154">
+        <v>1.5</v>
+      </c>
+      <c r="J324" s="18">
+        <v>252.0</v>
+      </c>
+      <c r="K324" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24.5x19x13 cm</t>
+        </is>
+      </c>
+      <c r="L324" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">303</t>
+        </is>
+      </c>
+      <c r="M324" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">polipropylen</t>
+        </is>
+      </c>
     </row>
-    <row r="325" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A325" s="12"/>
-      <c r="B325" s="65"/>
-      <c r="C325" s="15"/>
-      <c r="D325" s="14"/>
-      <c r="E325" s="14"/>
-      <c r="F325" s="31"/>
-      <c r="G325" s="151"/>
-      <c r="H325" s="155"/>
-      <c r="I325" s="15"/>
-      <c r="J325" s="15"/>
-      <c r="K325" s="15"/>
-      <c r="L325" s="11"/>
-      <c r="M325" s="11"/>
-      <c r="N325" s="32"/>
-      <c r="O325" s="32"/>
-      <c r="P325" s="32"/>
-      <c r="Q325" s="90"/>
-      <c r="R325" s="90"/>
-      <c r="S325" s="90"/>
-      <c r="T325" s="90"/>
-      <c r="U325" s="90"/>
-      <c r="V325" s="90"/>
-      <c r="W325" s="90"/>
-      <c r="X325" s="90"/>
-      <c r="Y325" s="90"/>
-      <c r="Z325" s="90"/>
-      <c r="AA325" s="90"/>
-      <c r="AB325" s="90"/>
-      <c r="AC325" s="90"/>
-      <c r="AD325" s="90"/>
-      <c r="AE325" s="90"/>
-      <c r="AF325" s="90"/>
-      <c r="AG325" s="90"/>
-      <c r="AH325" s="90"/>
-      <c r="AI325" s="90"/>
-      <c r="AJ325" s="90"/>
-      <c r="AK325" s="90"/>
-      <c r="AL325" s="90"/>
-      <c r="AM325" s="90"/>
-      <c r="AN325" s="90"/>
-      <c r="AO325" s="90"/>
-      <c r="AP325" s="90"/>
-      <c r="AQ325" s="90"/>
-      <c r="AR325" s="90"/>
-      <c r="AS325" s="90"/>
-      <c r="AT325" s="90"/>
-      <c r="AU325" s="90"/>
-      <c r="AV325" s="90"/>
-      <c r="AW325" s="90"/>
-      <c r="AX325" s="90"/>
+    <row r="325" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
+      <c r="A325" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">473.</t>
+        </is>
+      </c>
+      <c r="E325" s="20">
+        <v>5903456119560.0</v>
+      </c>
+      <c r="G325" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bio-waste container 6L BINI grey</t>
+        </is>
+      </c>
+      <c r="H325" s="154">
+        <v>1.8</v>
+      </c>
+      <c r="J325" s="18">
+        <v>162.0</v>
+      </c>
+      <c r="K325" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24.5x19x17,5 cm</t>
+        </is>
+      </c>
+      <c r="L325" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">333</t>
+        </is>
+      </c>
+      <c r="M325" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">polipropylen</t>
+        </is>
+      </c>
     </row>
-    <row r="326" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A326" s="12"/>
-      <c r="B326" s="65"/>
-      <c r="C326" s="15"/>
-      <c r="D326" s="14"/>
-      <c r="E326" s="14"/>
-      <c r="F326" s="31"/>
-      <c r="G326" s="151"/>
-      <c r="H326" s="155"/>
-      <c r="I326" s="15"/>
-      <c r="J326" s="15"/>
-      <c r="K326" s="15"/>
-      <c r="L326" s="11"/>
-      <c r="M326" s="11"/>
-      <c r="N326" s="32"/>
-      <c r="O326" s="32"/>
-      <c r="P326" s="32"/>
-      <c r="Q326" s="90"/>
-      <c r="R326" s="90"/>
-      <c r="S326" s="90"/>
-      <c r="T326" s="90"/>
-      <c r="U326" s="90"/>
-      <c r="V326" s="90"/>
-      <c r="W326" s="90"/>
-      <c r="X326" s="90"/>
-      <c r="Y326" s="90"/>
-      <c r="Z326" s="90"/>
-      <c r="AA326" s="90"/>
-      <c r="AB326" s="90"/>
-      <c r="AC326" s="90"/>
-      <c r="AD326" s="90"/>
-      <c r="AE326" s="90"/>
-      <c r="AF326" s="90"/>
-      <c r="AG326" s="90"/>
-      <c r="AH326" s="90"/>
-      <c r="AI326" s="90"/>
-      <c r="AJ326" s="90"/>
-      <c r="AK326" s="90"/>
-      <c r="AL326" s="90"/>
-      <c r="AM326" s="90"/>
-      <c r="AN326" s="90"/>
-      <c r="AO326" s="90"/>
-      <c r="AP326" s="90"/>
-      <c r="AQ326" s="90"/>
-      <c r="AR326" s="90"/>
-      <c r="AS326" s="90"/>
-      <c r="AT326" s="90"/>
-      <c r="AU326" s="90"/>
-      <c r="AV326" s="90"/>
-      <c r="AW326" s="90"/>
-      <c r="AX326" s="90"/>
+    <row r="326" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
+      <c r="A326" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">474.</t>
+        </is>
+      </c>
+      <c r="E326" s="20">
+        <v>5903456122928.0</v>
+      </c>
+      <c r="G326" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BINI BASIC set of 3 black waste segregation bins with color lid and color flap blue/green/yellow</t>
+        </is>
+      </c>
+      <c r="H326" s="154">
+        <v>10.5</v>
+      </c>
+      <c r="I326" s="18">
+        <v>1.0</v>
+      </c>
+      <c r="J326" s="18">
+        <v>27.0</v>
+      </c>
+      <c r="K326" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">54x25X39 cm</t>
+        </is>
+      </c>
+      <c r="L326" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3000</t>
+        </is>
+      </c>
+      <c r="M326" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">polipropylen</t>
+        </is>
+      </c>
     </row>
-    <row r="327" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A327" s="12"/>
-      <c r="B327" s="65"/>
-      <c r="C327" s="15"/>
-      <c r="D327" s="14"/>
-      <c r="E327" s="14"/>
-      <c r="F327" s="31"/>
-      <c r="G327" s="151"/>
-      <c r="H327" s="155"/>
-      <c r="I327" s="15"/>
-      <c r="J327" s="15"/>
-      <c r="K327" s="15"/>
-      <c r="L327" s="11"/>
-      <c r="M327" s="11"/>
-      <c r="N327" s="32"/>
-      <c r="O327" s="32"/>
-      <c r="P327" s="32"/>
-      <c r="Q327" s="90"/>
-      <c r="R327" s="90"/>
-      <c r="S327" s="90"/>
-      <c r="T327" s="90"/>
-      <c r="U327" s="90"/>
-      <c r="V327" s="90"/>
-      <c r="W327" s="90"/>
-      <c r="X327" s="90"/>
-      <c r="Y327" s="90"/>
-      <c r="Z327" s="90"/>
-      <c r="AA327" s="90"/>
-      <c r="AB327" s="90"/>
-      <c r="AC327" s="90"/>
-      <c r="AD327" s="90"/>
-      <c r="AE327" s="90"/>
-      <c r="AF327" s="90"/>
-      <c r="AG327" s="90"/>
-      <c r="AH327" s="90"/>
-      <c r="AI327" s="90"/>
-      <c r="AJ327" s="90"/>
-      <c r="AK327" s="90"/>
-      <c r="AL327" s="90"/>
-      <c r="AM327" s="90"/>
-      <c r="AN327" s="90"/>
-      <c r="AO327" s="90"/>
-      <c r="AP327" s="90"/>
-      <c r="AQ327" s="90"/>
-      <c r="AR327" s="90"/>
-      <c r="AS327" s="90"/>
-      <c r="AT327" s="90"/>
-      <c r="AU327" s="90"/>
-      <c r="AV327" s="90"/>
-      <c r="AW327" s="90"/>
-      <c r="AX327" s="90"/>
+    <row r="327" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
+      <c r="A327" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">475.</t>
+        </is>
+      </c>
+      <c r="E327" s="20">
+        <v>5903456123369.0</v>
+      </c>
+      <c r="G327" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">non-slip chopping board size M - mint</t>
+        </is>
+      </c>
+      <c r="H327" s="154">
+        <v>1.2646878355576012</v>
+      </c>
+      <c r="I327" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="J327" s="18">
+        <v>2800.0</v>
+      </c>
+      <c r="K327" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30x20x0.6 cm</t>
+        </is>
+      </c>
+      <c r="L327" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">259</t>
+        </is>
+      </c>
+      <c r="M327" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">polipropylen</t>
+        </is>
+      </c>
     </row>
-    <row r="328" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A328" s="12"/>
-      <c r="B328" s="65"/>
-      <c r="C328" s="15"/>
-      <c r="D328" s="14"/>
-      <c r="E328" s="14"/>
-      <c r="F328" s="31"/>
-      <c r="G328" s="151"/>
-      <c r="H328" s="155"/>
-      <c r="I328" s="15"/>
-      <c r="J328" s="15"/>
-      <c r="K328" s="15"/>
-      <c r="L328" s="11"/>
-      <c r="M328" s="11"/>
-      <c r="N328" s="32"/>
-      <c r="O328" s="32"/>
-      <c r="P328" s="32"/>
-      <c r="Q328" s="90"/>
-      <c r="R328" s="90"/>
-      <c r="S328" s="90"/>
-      <c r="T328" s="90"/>
-      <c r="U328" s="90"/>
-      <c r="V328" s="90"/>
-      <c r="W328" s="90"/>
-      <c r="X328" s="90"/>
-      <c r="Y328" s="90"/>
-      <c r="Z328" s="90"/>
-      <c r="AA328" s="90"/>
-      <c r="AB328" s="90"/>
-      <c r="AC328" s="90"/>
-      <c r="AD328" s="90"/>
-      <c r="AE328" s="90"/>
-      <c r="AF328" s="90"/>
-      <c r="AG328" s="90"/>
-      <c r="AH328" s="90"/>
-      <c r="AI328" s="90"/>
-      <c r="AJ328" s="90"/>
-      <c r="AK328" s="90"/>
-      <c r="AL328" s="90"/>
-      <c r="AM328" s="90"/>
-      <c r="AN328" s="90"/>
-      <c r="AO328" s="90"/>
-      <c r="AP328" s="90"/>
-      <c r="AQ328" s="90"/>
-      <c r="AR328" s="90"/>
-      <c r="AS328" s="90"/>
-      <c r="AT328" s="90"/>
-      <c r="AU328" s="90"/>
-      <c r="AV328" s="90"/>
-      <c r="AW328" s="90"/>
-      <c r="AX328" s="90"/>
+    <row r="328" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
+      <c r="A328" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">476.</t>
+        </is>
+      </c>
+      <c r="E328" s="20">
+        <v>5903456123390.0</v>
+      </c>
+      <c r="G328" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">non-slip chopping board size L - cappucino</t>
+        </is>
+      </c>
+      <c r="H328" s="154">
+        <v>1.7785243135450222</v>
+      </c>
+      <c r="I328" s="18">
+        <v>20.0</v>
+      </c>
+      <c r="J328" s="18">
+        <v>1400.0</v>
+      </c>
+      <c r="K328" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35x24x0.7 cm</t>
+        </is>
+      </c>
+      <c r="L328" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">501</t>
+        </is>
+      </c>
+      <c r="M328" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">polipropylen</t>
+        </is>
+      </c>
     </row>
-    <row r="329" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A329" s="12"/>
-      <c r="B329" s="65"/>
-      <c r="C329" s="15"/>
-      <c r="D329" s="14"/>
-      <c r="E329" s="14"/>
-      <c r="F329" s="31"/>
-      <c r="G329" s="151"/>
-      <c r="H329" s="155"/>
-      <c r="I329" s="15"/>
-      <c r="J329" s="15"/>
-      <c r="K329" s="15"/>
-      <c r="L329" s="11"/>
-      <c r="M329" s="11"/>
-      <c r="N329" s="32"/>
-      <c r="O329" s="32"/>
-      <c r="P329" s="32"/>
-      <c r="Q329" s="90"/>
-      <c r="R329" s="90"/>
-      <c r="S329" s="90"/>
-      <c r="T329" s="90"/>
-      <c r="U329" s="90"/>
-      <c r="V329" s="90"/>
-      <c r="W329" s="90"/>
-      <c r="X329" s="90"/>
-      <c r="Y329" s="90"/>
-      <c r="Z329" s="90"/>
-      <c r="AA329" s="90"/>
-      <c r="AB329" s="90"/>
-      <c r="AC329" s="90"/>
-      <c r="AD329" s="90"/>
-      <c r="AE329" s="90"/>
-      <c r="AF329" s="90"/>
-      <c r="AG329" s="90"/>
-      <c r="AH329" s="90"/>
-      <c r="AI329" s="90"/>
-      <c r="AJ329" s="90"/>
-      <c r="AK329" s="90"/>
-      <c r="AL329" s="90"/>
-      <c r="AM329" s="90"/>
-      <c r="AN329" s="90"/>
-      <c r="AO329" s="90"/>
-      <c r="AP329" s="90"/>
-      <c r="AQ329" s="90"/>
-      <c r="AR329" s="90"/>
-      <c r="AS329" s="90"/>
-      <c r="AT329" s="90"/>
-      <c r="AU329" s="90"/>
-      <c r="AV329" s="90"/>
-      <c r="AW329" s="90"/>
-      <c r="AX329" s="90"/>
+    <row r="329" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
+      <c r="A329" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">477.</t>
+        </is>
+      </c>
+      <c r="E329" s="20">
+        <v>5903456119065.0</v>
+      </c>
+      <c r="G329" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Food container 1 l</t>
+        </is>
+      </c>
+      <c r="H329" s="154">
+        <v>0.9064095292115713</v>
+      </c>
+      <c r="I329" s="18">
+        <v>8.0</v>
+      </c>
+      <c r="J329" s="18">
+        <v>560.0</v>
+      </c>
+      <c r="K329" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20x14x7 cm</t>
+        </is>
+      </c>
+      <c r="L329" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">150</t>
+        </is>
+      </c>
+      <c r="M329" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">polipropylen,silikon</t>
+        </is>
+      </c>
     </row>
-    <row r="330" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A330" s="12"/>
-      <c r="B330" s="65"/>
-      <c r="C330" s="15"/>
-      <c r="D330" s="14"/>
-      <c r="E330" s="14"/>
-      <c r="F330" s="31"/>
-      <c r="G330" s="151"/>
-      <c r="H330" s="155"/>
-      <c r="I330" s="15"/>
-      <c r="J330" s="15"/>
-      <c r="K330" s="15"/>
-      <c r="L330" s="11"/>
-      <c r="M330" s="11"/>
-      <c r="N330" s="32"/>
-      <c r="O330" s="32"/>
-      <c r="P330" s="32"/>
-      <c r="Q330" s="90"/>
-      <c r="R330" s="90"/>
-      <c r="S330" s="90"/>
-      <c r="T330" s="90"/>
-      <c r="U330" s="90"/>
-      <c r="V330" s="90"/>
-      <c r="W330" s="90"/>
-      <c r="X330" s="90"/>
-      <c r="Y330" s="90"/>
-      <c r="Z330" s="90"/>
-      <c r="AA330" s="90"/>
-      <c r="AB330" s="90"/>
-      <c r="AC330" s="90"/>
-      <c r="AD330" s="90"/>
-      <c r="AE330" s="90"/>
-      <c r="AF330" s="90"/>
-      <c r="AG330" s="90"/>
-      <c r="AH330" s="90"/>
-      <c r="AI330" s="90"/>
-      <c r="AJ330" s="90"/>
-      <c r="AK330" s="90"/>
-      <c r="AL330" s="90"/>
-      <c r="AM330" s="90"/>
-      <c r="AN330" s="90"/>
-      <c r="AO330" s="90"/>
-      <c r="AP330" s="90"/>
-      <c r="AQ330" s="90"/>
-      <c r="AR330" s="90"/>
-      <c r="AS330" s="90"/>
-      <c r="AT330" s="90"/>
-      <c r="AU330" s="90"/>
-      <c r="AV330" s="90"/>
-      <c r="AW330" s="90"/>
-      <c r="AX330" s="90"/>
+    <row r="330" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
+      <c r="A330" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">478.</t>
+        </is>
+      </c>
+      <c r="E330" s="20">
+        <v>5903456123246.0</v>
+      </c>
+      <c r="G330" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bowl with 2 grinders - MINT</t>
+        </is>
+      </c>
+      <c r="H330" s="154">
+        <v>2.3920846755637366</v>
+      </c>
+      <c r="I330" s="18">
+        <v>6.0</v>
+      </c>
+      <c r="J330" s="18">
+        <v>162.0</v>
+      </c>
+      <c r="K330" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24x29x14,5cm</t>
+        </is>
+      </c>
+      <c r="L330" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">430</t>
+        </is>
+      </c>
+      <c r="M330" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">polipropylen</t>
+        </is>
+      </c>
     </row>
-    <row r="331" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A331" s="12"/>
-      <c r="B331" s="65"/>
-      <c r="C331" s="15"/>
-      <c r="D331" s="14"/>
-      <c r="E331" s="14"/>
-      <c r="F331" s="31"/>
-      <c r="G331" s="151"/>
-      <c r="H331" s="155"/>
-      <c r="I331" s="15"/>
-      <c r="J331" s="15"/>
-      <c r="K331" s="15"/>
-      <c r="L331" s="11"/>
-      <c r="M331" s="11"/>
-      <c r="N331" s="32"/>
-      <c r="O331" s="32"/>
-      <c r="P331" s="32"/>
-      <c r="Q331" s="90"/>
-      <c r="R331" s="90"/>
-      <c r="S331" s="90"/>
-      <c r="T331" s="90"/>
-      <c r="U331" s="90"/>
-      <c r="V331" s="90"/>
-      <c r="W331" s="90"/>
-      <c r="X331" s="90"/>
-      <c r="Y331" s="90"/>
-      <c r="Z331" s="90"/>
-      <c r="AA331" s="90"/>
-      <c r="AB331" s="90"/>
-      <c r="AC331" s="90"/>
-      <c r="AD331" s="90"/>
-      <c r="AE331" s="90"/>
-      <c r="AF331" s="90"/>
-      <c r="AG331" s="90"/>
-      <c r="AH331" s="90"/>
-      <c r="AI331" s="90"/>
-      <c r="AJ331" s="90"/>
-      <c r="AK331" s="90"/>
-      <c r="AL331" s="90"/>
-      <c r="AM331" s="90"/>
-      <c r="AN331" s="90"/>
-      <c r="AO331" s="90"/>
-      <c r="AP331" s="90"/>
-      <c r="AQ331" s="90"/>
-      <c r="AR331" s="90"/>
-      <c r="AS331" s="90"/>
-      <c r="AT331" s="90"/>
-      <c r="AU331" s="90"/>
-      <c r="AV331" s="90"/>
-      <c r="AW331" s="90"/>
-      <c r="AX331" s="90"/>
+    <row r="331" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
+      <c r="A331" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">479.</t>
+        </is>
+      </c>
+      <c r="E331" s="20">
+        <v>5903456123765.0</v>
+      </c>
+      <c r="G331" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Container for loose products,  0,65 l</t>
+        </is>
+      </c>
+      <c r="H331" s="154">
+        <v>0.6741064580457127</v>
+      </c>
+      <c r="I331" s="18">
+        <v>12.0</v>
+      </c>
+      <c r="J331" s="18">
+        <v>840.0</v>
+      </c>
+      <c r="K331" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10x10,5x10,5 cm</t>
+        </is>
+      </c>
+      <c r="L331" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">162</t>
+        </is>
+      </c>
+      <c r="M331" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PET, silikon</t>
+        </is>
+      </c>
     </row>
-    <row r="332" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A332" s="12"/>
-      <c r="B332" s="65"/>
-      <c r="C332" s="15"/>
-      <c r="D332" s="14"/>
-      <c r="E332" s="14"/>
-      <c r="F332" s="31"/>
-      <c r="G332" s="151"/>
-      <c r="H332" s="155"/>
-      <c r="I332" s="15"/>
-      <c r="J332" s="15"/>
-      <c r="K332" s="15"/>
-      <c r="L332" s="11"/>
-      <c r="M332" s="11"/>
-      <c r="N332" s="32"/>
-      <c r="O332" s="32"/>
-      <c r="P332" s="32"/>
-      <c r="Q332" s="90"/>
-      <c r="R332" s="90"/>
-      <c r="S332" s="90"/>
-      <c r="T332" s="90"/>
-      <c r="U332" s="90"/>
-      <c r="V332" s="90"/>
-      <c r="W332" s="90"/>
-      <c r="X332" s="90"/>
-      <c r="Y332" s="90"/>
-      <c r="Z332" s="90"/>
-      <c r="AA332" s="90"/>
-      <c r="AB332" s="90"/>
-      <c r="AC332" s="90"/>
-      <c r="AD332" s="90"/>
-      <c r="AE332" s="90"/>
-      <c r="AF332" s="90"/>
-      <c r="AG332" s="90"/>
-      <c r="AH332" s="90"/>
-      <c r="AI332" s="90"/>
-      <c r="AJ332" s="90"/>
-      <c r="AK332" s="90"/>
-      <c r="AL332" s="90"/>
-      <c r="AM332" s="90"/>
-      <c r="AN332" s="90"/>
-      <c r="AO332" s="90"/>
-      <c r="AP332" s="90"/>
-      <c r="AQ332" s="90"/>
-      <c r="AR332" s="90"/>
-      <c r="AS332" s="90"/>
-      <c r="AT332" s="90"/>
-      <c r="AU332" s="90"/>
-      <c r="AV332" s="90"/>
-      <c r="AW332" s="90"/>
-      <c r="AX332" s="90"/>
+    <row r="332" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
+      <c r="A332" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">480.</t>
+        </is>
+      </c>
+      <c r="E332" s="20">
+        <v>5903456123772.0</v>
+      </c>
+      <c r="G332" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Container for loose products, 0,9 l</t>
+        </is>
+      </c>
+      <c r="H332" s="154">
+        <v>0.8510130339398634</v>
+      </c>
+      <c r="I332" s="18">
+        <v>12.0</v>
+      </c>
+      <c r="J332" s="18">
+        <v>840.0</v>
+      </c>
+      <c r="K332" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14x10,5x10,5cm</t>
+        </is>
+      </c>
+      <c r="L332" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">199</t>
+        </is>
+      </c>
+      <c r="M332" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PET, silikon</t>
+        </is>
+      </c>
     </row>
-    <row r="333" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A333" s="12"/>
-      <c r="B333" s="65"/>
-      <c r="C333" s="15"/>
-      <c r="D333" s="14"/>
-      <c r="E333" s="14"/>
-      <c r="F333" s="31"/>
-      <c r="G333" s="151"/>
-      <c r="H333" s="155"/>
-      <c r="I333" s="15"/>
-      <c r="J333" s="15"/>
-      <c r="K333" s="15"/>
-      <c r="L333" s="11"/>
-      <c r="M333" s="11"/>
-      <c r="N333" s="32"/>
-      <c r="O333" s="32"/>
-      <c r="P333" s="32"/>
-      <c r="Q333" s="90"/>
-      <c r="R333" s="90"/>
-      <c r="S333" s="90"/>
-      <c r="T333" s="90"/>
-      <c r="U333" s="90"/>
-      <c r="V333" s="90"/>
-      <c r="W333" s="90"/>
-      <c r="X333" s="90"/>
-      <c r="Y333" s="90"/>
-      <c r="Z333" s="90"/>
-      <c r="AA333" s="90"/>
-      <c r="AB333" s="90"/>
-      <c r="AC333" s="90"/>
-      <c r="AD333" s="90"/>
-      <c r="AE333" s="90"/>
-      <c r="AF333" s="90"/>
-      <c r="AG333" s="90"/>
-      <c r="AH333" s="90"/>
-      <c r="AI333" s="90"/>
-      <c r="AJ333" s="90"/>
-      <c r="AK333" s="90"/>
-      <c r="AL333" s="90"/>
-      <c r="AM333" s="90"/>
-      <c r="AN333" s="90"/>
-      <c r="AO333" s="90"/>
-      <c r="AP333" s="90"/>
-      <c r="AQ333" s="90"/>
-      <c r="AR333" s="90"/>
-      <c r="AS333" s="90"/>
-      <c r="AT333" s="90"/>
-      <c r="AU333" s="90"/>
-      <c r="AV333" s="90"/>
-      <c r="AW333" s="90"/>
-      <c r="AX333" s="90"/>
+    <row r="333" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
+      <c r="A333" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">481.</t>
+        </is>
+      </c>
+      <c r="E333" s="20">
+        <v>5903456123789.0</v>
+      </c>
+      <c r="G333" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Container for loose products, 1,6 l</t>
+        </is>
+      </c>
+      <c r="H333" s="154">
+        <v>0.9794520547945206</v>
+      </c>
+      <c r="I333" s="18">
+        <v>12.0</v>
+      </c>
+      <c r="J333" s="18">
+        <v>480.0</v>
+      </c>
+      <c r="K333" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24x10,5x10,5 cm</t>
+        </is>
+      </c>
+      <c r="L333" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">296</t>
+        </is>
+      </c>
+      <c r="M333" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PET, silikon</t>
+        </is>
+      </c>
     </row>
     <row r="334" spans="1:123" s="17" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A334" s="12"/>
@@ -52292,429 +52143,6 @@
       <c r="AW422" s="90"/>
       <c r="AX422" s="90"/>
     </row>
-    <row r="323" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
-      <c r="A323" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">471.</t>
-        </is>
-      </c>
-      <c r="E323" s="20">
-        <v>5903456123697.0</v>
-      </c>
-      <c r="G323" s="136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Folding table for bed - cappuccino</t>
-        </is>
-      </c>
-      <c r="H323" s="154">
-        <v>4.2526942711287585</v>
-      </c>
-      <c r="I323" s="18">
-        <v>6.0</v>
-      </c>
-      <c r="J323" s="18">
-        <v>108.0</v>
-      </c>
-      <c r="K323" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">54x35.5x26 cm</t>
-        </is>
-      </c>
-      <c r="L323" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">970</t>
-        </is>
-      </c>
-      <c r="M323" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">polipropylen</t>
-        </is>
-      </c>
-    </row>
-    <row r="324" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
-      <c r="A324" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">472.</t>
-        </is>
-      </c>
-      <c r="E324" s="20">
-        <v>5903456119478.0</v>
-      </c>
-      <c r="G324" s="136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MINI BINI - handy container for bio waste - green color container gray cover 35% bio - 4.5L</t>
-        </is>
-      </c>
-      <c r="H324" s="154">
-        <v>1.5</v>
-      </c>
-      <c r="J324" s="18">
-        <v>252.0</v>
-      </c>
-      <c r="K324" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">24.5x19x13 cm</t>
-        </is>
-      </c>
-      <c r="L324" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">303</t>
-        </is>
-      </c>
-      <c r="M324" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">polipropylen</t>
-        </is>
-      </c>
-    </row>
-    <row r="325" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
-      <c r="A325" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">473.</t>
-        </is>
-      </c>
-      <c r="E325" s="20">
-        <v>5903456119560.0</v>
-      </c>
-      <c r="G325" s="136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bio-waste container 6L BINI grey</t>
-        </is>
-      </c>
-      <c r="H325" s="154">
-        <v>1.8</v>
-      </c>
-      <c r="J325" s="18">
-        <v>162.0</v>
-      </c>
-      <c r="K325" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">24.5x19x17,5 cm</t>
-        </is>
-      </c>
-      <c r="L325" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">333</t>
-        </is>
-      </c>
-      <c r="M325" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">polipropylen</t>
-        </is>
-      </c>
-    </row>
-    <row r="326" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
-      <c r="A326" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">474.</t>
-        </is>
-      </c>
-      <c r="E326" s="20">
-        <v>5903456122928.0</v>
-      </c>
-      <c r="G326" s="136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BINI BASIC set of 3 black waste segregation bins with color lid and color flap blue/green/yellow</t>
-        </is>
-      </c>
-      <c r="H326" s="154">
-        <v>10.5</v>
-      </c>
-      <c r="I326" s="18">
-        <v>1.0</v>
-      </c>
-      <c r="J326" s="18">
-        <v>27.0</v>
-      </c>
-      <c r="K326" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">54x25X39 cm</t>
-        </is>
-      </c>
-      <c r="L326" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3000</t>
-        </is>
-      </c>
-      <c r="M326" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">polipropylen</t>
-        </is>
-      </c>
-    </row>
-    <row r="327" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
-      <c r="A327" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">475.</t>
-        </is>
-      </c>
-      <c r="E327" s="20">
-        <v>5903456123369.0</v>
-      </c>
-      <c r="G327" s="136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">non-slip chopping board size M - mint</t>
-        </is>
-      </c>
-      <c r="H327" s="154">
-        <v>1.2646878355576012</v>
-      </c>
-      <c r="I327" s="18">
-        <v>40.0</v>
-      </c>
-      <c r="J327" s="18">
-        <v>2800.0</v>
-      </c>
-      <c r="K327" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30x20x0.6 cm</t>
-        </is>
-      </c>
-      <c r="L327" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">259</t>
-        </is>
-      </c>
-      <c r="M327" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">polipropylen</t>
-        </is>
-      </c>
-    </row>
-    <row r="328" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
-      <c r="A328" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">476.</t>
-        </is>
-      </c>
-      <c r="E328" s="20">
-        <v>5903456123390.0</v>
-      </c>
-      <c r="G328" s="136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">non-slip chopping board size L - cappucino</t>
-        </is>
-      </c>
-      <c r="H328" s="154">
-        <v>1.7785243135450222</v>
-      </c>
-      <c r="I328" s="18">
-        <v>20.0</v>
-      </c>
-      <c r="J328" s="18">
-        <v>1400.0</v>
-      </c>
-      <c r="K328" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">35x24x0.7 cm</t>
-        </is>
-      </c>
-      <c r="L328" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">501</t>
-        </is>
-      </c>
-      <c r="M328" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">polipropylen</t>
-        </is>
-      </c>
-    </row>
-    <row r="329" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
-      <c r="A329" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">477.</t>
-        </is>
-      </c>
-      <c r="E329" s="20">
-        <v>5903456119065.0</v>
-      </c>
-      <c r="G329" s="136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Food container 1 l</t>
-        </is>
-      </c>
-      <c r="H329" s="154">
-        <v>0.9064095292115713</v>
-      </c>
-      <c r="I329" s="18">
-        <v>8.0</v>
-      </c>
-      <c r="J329" s="18">
-        <v>560.0</v>
-      </c>
-      <c r="K329" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20x14x7 cm</t>
-        </is>
-      </c>
-      <c r="L329" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">150</t>
-        </is>
-      </c>
-      <c r="M329" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">polipropylen,silikon</t>
-        </is>
-      </c>
-    </row>
-    <row r="330" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
-      <c r="A330" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">478.</t>
-        </is>
-      </c>
-      <c r="E330" s="20">
-        <v>5903456123246.0</v>
-      </c>
-      <c r="G330" s="136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bowl with 2 grinders - MINT</t>
-        </is>
-      </c>
-      <c r="H330" s="154">
-        <v>2.3920846755637366</v>
-      </c>
-      <c r="I330" s="18">
-        <v>6.0</v>
-      </c>
-      <c r="J330" s="18">
-        <v>162.0</v>
-      </c>
-      <c r="K330" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">24x29x14,5cm</t>
-        </is>
-      </c>
-      <c r="L330" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">430</t>
-        </is>
-      </c>
-      <c r="M330" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">polipropylen</t>
-        </is>
-      </c>
-    </row>
-    <row r="331" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
-      <c r="A331" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">479.</t>
-        </is>
-      </c>
-      <c r="E331" s="20">
-        <v>5903456123765.0</v>
-      </c>
-      <c r="G331" s="136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Container for loose products,  0,65 l</t>
-        </is>
-      </c>
-      <c r="H331" s="154">
-        <v>0.6741064580457127</v>
-      </c>
-      <c r="I331" s="18">
-        <v>12.0</v>
-      </c>
-      <c r="J331" s="18">
-        <v>840.0</v>
-      </c>
-      <c r="K331" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10x10,5x10,5 cm</t>
-        </is>
-      </c>
-      <c r="L331" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">162</t>
-        </is>
-      </c>
-      <c r="M331" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PET, silikon</t>
-        </is>
-      </c>
-    </row>
-    <row r="332" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
-      <c r="A332" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">480.</t>
-        </is>
-      </c>
-      <c r="E332" s="20">
-        <v>5903456123772.0</v>
-      </c>
-      <c r="G332" s="136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Container for loose products, 0,9 l</t>
-        </is>
-      </c>
-      <c r="H332" s="154">
-        <v>0.8510130339398634</v>
-      </c>
-      <c r="I332" s="18">
-        <v>12.0</v>
-      </c>
-      <c r="J332" s="18">
-        <v>840.0</v>
-      </c>
-      <c r="K332" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14x10,5x10,5cm</t>
-        </is>
-      </c>
-      <c r="L332" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">199</t>
-        </is>
-      </c>
-      <c r="M332" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PET, silikon</t>
-        </is>
-      </c>
-    </row>
-    <row r="333" spans="1:51" s="16" customFormat="1" ht="153" customHeight="1">
-      <c r="A333" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">481.</t>
-        </is>
-      </c>
-      <c r="E333" s="20">
-        <v>5903456123789.0</v>
-      </c>
-      <c r="G333" s="136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Container for loose products, 1,6 l</t>
-        </is>
-      </c>
-      <c r="H333" s="154">
-        <v>0.9794520547945206</v>
-      </c>
-      <c r="I333" s="18">
-        <v>12.0</v>
-      </c>
-      <c r="J333" s="18">
-        <v>480.0</v>
-      </c>
-      <c r="K333" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">24x10,5x10,5 cm</t>
-        </is>
-      </c>
-      <c r="L333" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">296</t>
-        </is>
-      </c>
-      <c r="M333" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PET, silikon</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="25" type="noConversion"/>
   <conditionalFormatting sqref="B149">

</xml_diff>